<commit_message>
fix: update excel document
</commit_message>
<xml_diff>
--- a/sistema/HistóricoDoMeuExperimento.xlsx
+++ b/sistema/HistóricoDoMeuExperimento.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aliss\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aliss\Desktop\automated-test-generator\sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{21621BFB-EB00-422A-B493-CEA446E384E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81DE2AD-0529-4B55-BD2C-ECD0359C11C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -245,9 +245,6 @@
 Anexo: template de header.</t>
   </si>
   <si>
-    <t>Claude Sonnet 4.6 - Claude Code - Skills and Agents</t>
-  </si>
-  <si>
     <t xml:space="preserve">Com base nos testes anteriores, gere os testes para o proof, utilizando a skill @.agents/skills/cucumber-gherkin/SKILL.md  </t>
   </si>
   <si>
@@ -267,6 +264,9 @@
   </si>
   <si>
     <t>Criou corretamente a interface, gerando as informações de correção da prova conforme o esperado.</t>
+  </si>
+  <si>
+    <t>Claude Sonnet 4.6 - Claude Code - Skills: cucumber-gherkin, git-commit, nodejs-backend-patterns, vercel-react-best-practices and Agents: CLAUDE.md</t>
   </si>
 </sst>
 </file>
@@ -1675,7 +1675,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="27.6" customHeight="1">
       <c r="A1" s="13" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -2033,7 +2033,7 @@
         <v>14</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>17</v>
@@ -2041,7 +2041,7 @@
     </row>
     <row r="23" spans="1:5" ht="25.5">
       <c r="A23" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>17</v>
@@ -2050,7 +2050,7 @@
         <v>29</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>17</v>
@@ -2058,7 +2058,7 @@
     </row>
     <row r="24" spans="1:5" ht="76.5">
       <c r="A24" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>17</v>
@@ -2067,7 +2067,7 @@
         <v>14</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E24" s="9" t="s">
         <v>17</v>
@@ -2075,7 +2075,7 @@
     </row>
     <row r="25" spans="1:5" ht="63.75">
       <c r="A25" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>17</v>
@@ -2084,7 +2084,7 @@
         <v>14</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>17</v>

</xml_diff>